<commit_message>
complete full flow testing (API + UI) and update test cases with results and bugs ver2
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="121">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -194,9 +194,6 @@
     <t>Send POST /api/users with invalid data</t>
   </si>
   <si>
-    <t>Error 400</t>
-  </si>
-  <si>
     <t>BUG01</t>
   </si>
   <si>
@@ -381,6 +378,15 @@
   </si>
   <si>
     <t>Payment recorded successfully, invoice status updated accordingly</t>
+  </si>
+  <si>
+    <t>User created successfully with empty fields, no validation applied</t>
+  </si>
+  <si>
+    <t>Tenant created successfully, new tenant returned with id = X and correct data</t>
+  </si>
+  <si>
+    <t>Tenant created successfully</t>
   </si>
 </sst>
 </file>
@@ -444,7 +450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -462,7 +468,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -758,11 +763,11 @@
     <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.33203125" customWidth="1"/>
-    <col min="4" max="4" width="66.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.21875" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" style="9" customWidth="1"/>
-    <col min="8" max="8" width="28.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="85" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" style="8" customWidth="1"/>
+    <col min="8" max="8" width="28.21875" style="8" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="105.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
   </cols>
@@ -815,10 +820,10 @@
       <c r="E2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H2" s="3" t="s">
@@ -845,20 +850,20 @@
       <c r="E3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>50</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>53</v>
       </c>
       <c r="I3" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="21" x14ac:dyDescent="0.4">
@@ -872,15 +877,15 @@
         <v>36</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H4" s="3" t="s">
@@ -902,22 +907,22 @@
         <v>33</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>53</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J5" s="6"/>
     </row>
@@ -932,15 +937,15 @@
         <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H6" s="3" t="s">
@@ -962,15 +967,15 @@
         <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="G7" s="10" t="s">
+      <c r="F7" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H7" s="3" t="s">
@@ -992,25 +997,25 @@
         <v>13</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>50</v>
+      <c r="G8" s="9" t="s">
+        <v>43</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="J8" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="21" x14ac:dyDescent="0.4">
@@ -1024,15 +1029,15 @@
         <v>18</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="G9" s="10" t="s">
+      <c r="F9" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H9" s="3" t="s">
@@ -1054,22 +1059,22 @@
         <v>41</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>53</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J10" s="6"/>
     </row>
@@ -1084,15 +1089,15 @@
         <v>23</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="10" t="s">
+      <c r="F11" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G11" s="9" t="s">
         <v>43</v>
       </c>
       <c r="H11" s="3" t="s">
@@ -1114,25 +1119,25 @@
         <v>23</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="G12" s="10" t="s">
+      <c r="F12" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>50</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>53</v>
       </c>
       <c r="I12" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="21" x14ac:dyDescent="0.4">
@@ -1146,264 +1151,264 @@
         <v>29</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G13" s="10" t="s">
+      <c r="F13" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>50</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>53</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="F14" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H14" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>91</v>
-      </c>
       <c r="I14" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J14" s="6"/>
     </row>
     <row r="15" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="F15" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G15" s="8" t="s">
+      <c r="G15" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H15" s="8" t="s">
-        <v>91</v>
+      <c r="H15" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J15" s="6"/>
     </row>
     <row r="16" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>91</v>
+      <c r="F16" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J16" s="6"/>
     </row>
     <row r="17" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C17" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>91</v>
+      <c r="F17" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J17" s="6"/>
     </row>
     <row r="18" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C18" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>91</v>
+      <c r="F18" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J18" s="6"/>
     </row>
     <row r="19" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="C19" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="E19" s="7" t="s">
+      <c r="D19" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F19" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>91</v>
+      <c r="F19" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J19" s="6"/>
     </row>
     <row r="20" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="C20" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E20" s="7" t="s">
+      <c r="D20" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F20" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>91</v>
+      <c r="F20" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J20" s="6"/>
     </row>
     <row r="21" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C21" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E21" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>91</v>
+      <c r="F21" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J21" s="6"/>
     </row>

</xml_diff>